<commit_message>
BSD Mercedes - coduri unice cu V1 V2 V3
</commit_message>
<xml_diff>
--- a/BSD-Mercedes-Benz-Final.xlsx
+++ b/BSD-Mercedes-Benz-Final.xlsx
@@ -520,7 +520,7 @@
   <dimension ref="A1:F44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
     <col width="70" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
@@ -563,7 +563,7 @@
     <row r="2" ht="40" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>BSD-01+BSD-MB-01</t>
+          <t>BSD-01+BSD-MB-01-V1</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -587,7 +587,7 @@
     <row r="3" ht="40" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>BSD-01+BSD-MB-01</t>
+          <t>BSD-01+BSD-MB-01-V2</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -611,7 +611,7 @@
     <row r="4" ht="40" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>BSD-01+BSD-MB-01</t>
+          <t>BSD-01+BSD-MB-01-V3</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -635,7 +635,7 @@
     <row r="5" ht="40" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>BSD-01+BSD-MB-01</t>
+          <t>BSD-01+BSD-MB-01-V4</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -659,7 +659,7 @@
     <row r="6" ht="40" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>BSD-01+BSD-MB-01</t>
+          <t>BSD-01+BSD-MB-01-V5</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -683,7 +683,7 @@
     <row r="7" ht="40" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>BSD-01+BSD-MB-01</t>
+          <t>BSD-01+BSD-MB-01-V6</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -707,7 +707,7 @@
     <row r="8" ht="40" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>BSD-01+BSD-MB-01</t>
+          <t>BSD-01+BSD-MB-01-V7</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -731,7 +731,7 @@
     <row r="9" ht="40" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>BSD-01+BSD-MB-01</t>
+          <t>BSD-01+BSD-MB-01-V8</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -755,7 +755,7 @@
     <row r="10" ht="40" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>BSD-01+BSD-MB-01</t>
+          <t>BSD-01+BSD-MB-01-V9</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -779,7 +779,7 @@
     <row r="11" ht="40" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>BSD-01+BSD-MB-02</t>
+          <t>BSD-01+BSD-MB-02-V1</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
@@ -803,7 +803,7 @@
     <row r="12" ht="40" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>BSD-01+BSD-MB-02</t>
+          <t>BSD-01+BSD-MB-02-V2</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="13" ht="40" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>BSD-01+BSD-MB-02</t>
+          <t>BSD-01+BSD-MB-02-V3</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -851,7 +851,7 @@
     <row r="14" ht="40" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>BSD-01+BSD-MB-02</t>
+          <t>BSD-01+BSD-MB-02-V4</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
@@ -875,7 +875,7 @@
     <row r="15" ht="40" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>BSD-01+BSD-MB-02</t>
+          <t>BSD-01+BSD-MB-02-V5</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
@@ -899,7 +899,7 @@
     <row r="16" ht="40" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>BSD-01+BSD-MB-02</t>
+          <t>BSD-01+BSD-MB-02-V6</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
@@ -923,7 +923,7 @@
     <row r="17" ht="40" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>BSD-01+BSD-MB-03</t>
+          <t>BSD-01+BSD-MB-03-V1</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
@@ -947,7 +947,7 @@
     <row r="18" ht="40" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>BSD-01+BSD-MB-03</t>
+          <t>BSD-01+BSD-MB-03-V2</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
@@ -971,7 +971,7 @@
     <row r="19" ht="40" customHeight="1">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>BSD-01+BSD-MB-03</t>
+          <t>BSD-01+BSD-MB-03-V3</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
@@ -995,7 +995,7 @@
     <row r="20" ht="40" customHeight="1">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>BSD-01+BSD-MB-03</t>
+          <t>BSD-01+BSD-MB-03-V4</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
@@ -1019,7 +1019,7 @@
     <row r="21" ht="40" customHeight="1">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>BSD-01+BSD-MB-03</t>
+          <t>BSD-01+BSD-MB-03-V5</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
@@ -1043,7 +1043,7 @@
     <row r="22" ht="40" customHeight="1">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>BSD-01+BSD-MB-03</t>
+          <t>BSD-01+BSD-MB-03-V6</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
@@ -1067,7 +1067,7 @@
     <row r="23" ht="40" customHeight="1">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>BSD-01+BSD-MB-03</t>
+          <t>BSD-01+BSD-MB-03-V7</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
@@ -1091,7 +1091,7 @@
     <row r="24" ht="40" customHeight="1">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>BSD-01+BSD-MB-03</t>
+          <t>BSD-01+BSD-MB-03-V8</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
@@ -1115,7 +1115,7 @@
     <row r="25" ht="40" customHeight="1">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>BSD-01+BSD-MB-03</t>
+          <t>BSD-01+BSD-MB-03-V9</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
@@ -1139,7 +1139,7 @@
     <row r="26" ht="40" customHeight="1">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>BSD-01+BSD-MB-03</t>
+          <t>BSD-01+BSD-MB-03-V10</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
@@ -1163,7 +1163,7 @@
     <row r="27" ht="40" customHeight="1">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>BSD-01+BSD-MB-03</t>
+          <t>BSD-01+BSD-MB-03-V11</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
@@ -1187,7 +1187,7 @@
     <row r="28" ht="40" customHeight="1">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>BSD-01+BSD-MB-03</t>
+          <t>BSD-01+BSD-MB-03-V12</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
@@ -1211,7 +1211,7 @@
     <row r="29" ht="40" customHeight="1">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>BSD-01+BSD-MB-04</t>
+          <t>BSD-01+BSD-MB-04-V1</t>
         </is>
       </c>
       <c r="B29" s="9" t="inlineStr">
@@ -1235,7 +1235,7 @@
     <row r="30" ht="40" customHeight="1">
       <c r="A30" s="8" t="inlineStr">
         <is>
-          <t>BSD-01+BSD-MB-04</t>
+          <t>BSD-01+BSD-MB-04-V2</t>
         </is>
       </c>
       <c r="B30" s="9" t="inlineStr">
@@ -1259,7 +1259,7 @@
     <row r="31" ht="40" customHeight="1">
       <c r="A31" s="10" t="inlineStr">
         <is>
-          <t>BSD-01+BSD-MB-05</t>
+          <t>BSD-01+BSD-MB-05-V1</t>
         </is>
       </c>
       <c r="B31" s="11" t="inlineStr">
@@ -1283,7 +1283,7 @@
     <row r="32" ht="40" customHeight="1">
       <c r="A32" s="10" t="inlineStr">
         <is>
-          <t>BSD-01+BSD-MB-05</t>
+          <t>BSD-01+BSD-MB-05-V2</t>
         </is>
       </c>
       <c r="B32" s="11" t="inlineStr">
@@ -1307,7 +1307,7 @@
     <row r="33" ht="40" customHeight="1">
       <c r="A33" s="10" t="inlineStr">
         <is>
-          <t>BSD-01+BSD-MB-05</t>
+          <t>BSD-01+BSD-MB-05-V3</t>
         </is>
       </c>
       <c r="B33" s="11" t="inlineStr">
@@ -1331,7 +1331,7 @@
     <row r="34" ht="40" customHeight="1">
       <c r="A34" s="10" t="inlineStr">
         <is>
-          <t>BSD-01+BSD-MB-05</t>
+          <t>BSD-01+BSD-MB-05-V4</t>
         </is>
       </c>
       <c r="B34" s="11" t="inlineStr">
@@ -1355,7 +1355,7 @@
     <row r="35" ht="40" customHeight="1">
       <c r="A35" s="12" t="inlineStr">
         <is>
-          <t>BSD-01+BSD-MB-06</t>
+          <t>BSD-01+BSD-MB-06-V1</t>
         </is>
       </c>
       <c r="B35" s="13" t="inlineStr">
@@ -1379,7 +1379,7 @@
     <row r="36" ht="40" customHeight="1">
       <c r="A36" s="12" t="inlineStr">
         <is>
-          <t>BSD-01+BSD-MB-06</t>
+          <t>BSD-01+BSD-MB-06-V2</t>
         </is>
       </c>
       <c r="B36" s="13" t="inlineStr">
@@ -1403,7 +1403,7 @@
     <row r="37" ht="40" customHeight="1">
       <c r="A37" s="12" t="inlineStr">
         <is>
-          <t>BSD-01+BSD-MB-06</t>
+          <t>BSD-01+BSD-MB-06-V3</t>
         </is>
       </c>
       <c r="B37" s="13" t="inlineStr">
@@ -1427,7 +1427,7 @@
     <row r="38" ht="40" customHeight="1">
       <c r="A38" s="12" t="inlineStr">
         <is>
-          <t>BSD-01+BSD-MB-06</t>
+          <t>BSD-01+BSD-MB-06-V4</t>
         </is>
       </c>
       <c r="B38" s="13" t="inlineStr">
@@ -1451,7 +1451,7 @@
     <row r="39" ht="40" customHeight="1">
       <c r="A39" s="12" t="inlineStr">
         <is>
-          <t>BSD-01+BSD-MB-06</t>
+          <t>BSD-01+BSD-MB-06-V5</t>
         </is>
       </c>
       <c r="B39" s="13" t="inlineStr">
@@ -1475,7 +1475,7 @@
     <row r="40" ht="40" customHeight="1">
       <c r="A40" s="12" t="inlineStr">
         <is>
-          <t>BSD-01+BSD-MB-06</t>
+          <t>BSD-01+BSD-MB-06-V6</t>
         </is>
       </c>
       <c r="B40" s="13" t="inlineStr">
@@ -1499,7 +1499,7 @@
     <row r="41" ht="40" customHeight="1">
       <c r="A41" s="12" t="inlineStr">
         <is>
-          <t>BSD-01+BSD-MB-06</t>
+          <t>BSD-01+BSD-MB-06-V7</t>
         </is>
       </c>
       <c r="B41" s="13" t="inlineStr">
@@ -1523,7 +1523,7 @@
     <row r="42" ht="40" customHeight="1">
       <c r="A42" s="14" t="inlineStr">
         <is>
-          <t>BSD-01+BSD-MB-07</t>
+          <t>BSD-01+BSD-MB-07-V1</t>
         </is>
       </c>
       <c r="B42" s="15" t="inlineStr">
@@ -1547,7 +1547,7 @@
     <row r="43" ht="40" customHeight="1">
       <c r="A43" s="14" t="inlineStr">
         <is>
-          <t>BSD-01+BSD-MB-07</t>
+          <t>BSD-01+BSD-MB-07-V2</t>
         </is>
       </c>
       <c r="B43" s="15" t="inlineStr">
@@ -1571,7 +1571,7 @@
     <row r="44" ht="40" customHeight="1">
       <c r="A44" s="14" t="inlineStr">
         <is>
-          <t>BSD-01+BSD-MB-07</t>
+          <t>BSD-01+BSD-MB-07-V3</t>
         </is>
       </c>
       <c r="B44" s="15" t="inlineStr">

</xml_diff>

<commit_message>
BSD Mercedes - atribute marca/model + titlu SEO
</commit_message>
<xml_diff>
--- a/BSD-Mercedes-Benz-Final.xlsx
+++ b/BSD-Mercedes-Benz-Final.xlsx
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F44"/>
+  <dimension ref="A1:H44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -526,6 +526,8 @@
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="35" customHeight="1">
@@ -536,7 +538,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Denumire Produs</t>
+          <t>Denumire Produs (SEO)</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -557,6 +559,16 @@
       <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Cod Set Oglinzi</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Marca (Atribut)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Model (Atribut)</t>
         </is>
       </c>
     </row>
@@ -568,7 +580,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Sistem unghi mort Mercedes dedicat cu oglinzi dedicate C-Class W204 2009-2014</t>
+          <t>Unghi mort Mercedes C-Class W204 2009-2014 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr"/>
@@ -583,6 +595,16 @@
           <t>BSD-MB-01</t>
         </is>
       </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>C-Class (W204) 2009-2014</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="40" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
@@ -592,7 +614,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Sistem unghi mort Mercedes dedicat cu oglinzi dedicate E-Class W212 2010-2015</t>
+          <t>Unghi mort Mercedes E-Class W212 2010-2015 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr"/>
@@ -607,6 +629,16 @@
           <t>BSD-MB-01</t>
         </is>
       </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>E-Class (W212) 2010-2015</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="40" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -616,7 +648,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Sistem unghi mort Mercedes dedicat cu oglinzi dedicate GLK W204 2009-2015</t>
+          <t>Unghi mort Mercedes GLK W204 2009-2015 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr"/>
@@ -631,6 +663,16 @@
           <t>BSD-MB-01</t>
         </is>
       </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>GLK (W204) 2009-2015</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="40" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
@@ -640,7 +682,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Sistem unghi mort Mercedes dedicat cu oglinzi dedicate GLA X156 2015-2019</t>
+          <t>Unghi mort Mercedes GLA X156 2015-2019 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr"/>
@@ -655,6 +697,16 @@
           <t>BSD-MB-01</t>
         </is>
       </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>GLA (X156) 2015-2019</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="40" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -664,7 +716,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Sistem unghi mort Mercedes dedicat cu oglinzi dedicate A-Class W176 2013-2018</t>
+          <t>Unghi mort Mercedes A-Class W176 2013-2018 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr"/>
@@ -679,6 +731,16 @@
           <t>BSD-MB-01</t>
         </is>
       </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>A-Class (W176) 2013-2018</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="40" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
@@ -688,7 +750,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Sistem unghi mort Mercedes dedicat cu oglinzi dedicate B-Class W246 2012-2019</t>
+          <t>Unghi mort Mercedes B-Class W246 2012-2019 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr"/>
@@ -703,6 +765,16 @@
           <t>BSD-MB-01</t>
         </is>
       </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>B-Class (W246) 2012-2019</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="40" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -712,7 +784,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Sistem unghi mort Mercedes dedicat cu oglinzi dedicate CLA W117 2014-2019</t>
+          <t>Unghi mort Mercedes CLA W117 2014-2019 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr"/>
@@ -727,6 +799,16 @@
           <t>BSD-MB-01</t>
         </is>
       </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>CLA (W117) 2014-2019</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="40" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
@@ -736,7 +818,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Sistem unghi mort Mercedes dedicat cu oglinzi dedicate S-Class W221 2010-2013</t>
+          <t>Unghi mort Mercedes S-Class W221 2010-2013 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr"/>
@@ -751,6 +833,16 @@
           <t>BSD-MB-01</t>
         </is>
       </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>S-Class (W221) 2010-2013</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="40" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
@@ -760,7 +852,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Sistem unghi mort Mercedes dedicat cu oglinzi dedicate CLS W218 2011-2017</t>
+          <t>Unghi mort Mercedes CLS W218 2011-2017 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr"/>
@@ -775,6 +867,16 @@
           <t>BSD-MB-01</t>
         </is>
       </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>CLS (W218) 2011-2017</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="40" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
@@ -784,7 +886,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Sistem unghi mort Mercedes dedicat cu oglinzi dedicate ML W164 2010-2015</t>
+          <t>Unghi mort Mercedes ML W164 2010-2015 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr"/>
@@ -799,6 +901,16 @@
           <t>BSD-MB-02</t>
         </is>
       </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>ML (W164) 2010-2015</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="40" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
@@ -808,7 +920,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Sistem unghi mort Mercedes dedicat cu oglinzi dedicate GLE W166 2015-2019</t>
+          <t>Unghi mort Mercedes GLE W166 2015-2019 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr"/>
@@ -823,6 +935,16 @@
           <t>BSD-MB-02</t>
         </is>
       </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>GLE (W166) 2015-2019</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="40" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
@@ -832,7 +954,7 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Sistem unghi mort Mercedes dedicat cu oglinzi dedicate GLS X166 2016-2019</t>
+          <t>Unghi mort Mercedes GLS X166 2016-2019 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr"/>
@@ -847,6 +969,16 @@
           <t>BSD-MB-02</t>
         </is>
       </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>GLS (X166) 2016-2019</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="40" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
@@ -856,7 +988,7 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Sistem unghi mort Mercedes dedicat cu oglinzi dedicate GL X166 2013-2016</t>
+          <t>Unghi mort Mercedes GL X166 2013-2016 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr"/>
@@ -871,6 +1003,16 @@
           <t>BSD-MB-02</t>
         </is>
       </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>GL (X166) 2013-2016</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="40" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
@@ -880,7 +1022,7 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Sistem unghi mort Mercedes dedicat cu oglinzi dedicate R-Class W251 2009-2017</t>
+          <t>Unghi mort Mercedes R-Class W251 2009-2017 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr"/>
@@ -895,6 +1037,16 @@
           <t>BSD-MB-02</t>
         </is>
       </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>R-Class (W251) 2009-2017</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="40" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
@@ -904,7 +1056,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Sistem unghi mort Mercedes dedicat cu oglinzi dedicate G-Class W463 2013-2018</t>
+          <t>Unghi mort Mercedes G-Class W463 2013-2018 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr"/>
@@ -919,6 +1071,16 @@
           <t>BSD-MB-02</t>
         </is>
       </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>G-Class (W463) 2013-2018</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="40" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
@@ -928,7 +1090,7 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Sistem unghi mort Mercedes dedicat cu oglinzi dedicate C-Class W205 2015-2021</t>
+          <t>Unghi mort Mercedes C-Class W205 2015-2021 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr"/>
@@ -943,6 +1105,16 @@
           <t>BSD-MB-03</t>
         </is>
       </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>C-Class (W205) 2015-2021</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="40" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
@@ -952,7 +1124,7 @@
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Sistem unghi mort Mercedes dedicat cu oglinzi dedicate E-Class W213 2016-2023</t>
+          <t>Unghi mort Mercedes E-Class W213 2016-2023 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr"/>
@@ -967,6 +1139,16 @@
           <t>BSD-MB-03</t>
         </is>
       </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>E-Class (W213) 2016-2023</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="40" customHeight="1">
       <c r="A19" s="6" t="inlineStr">
@@ -976,7 +1158,7 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Sistem unghi mort Mercedes dedicat cu oglinzi dedicate GLA H247 2020-2024</t>
+          <t>Unghi mort Mercedes GLA H247 2020-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr"/>
@@ -991,6 +1173,16 @@
           <t>BSD-MB-03</t>
         </is>
       </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>GLA (H247) 2020-2024</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="40" customHeight="1">
       <c r="A20" s="6" t="inlineStr">
@@ -1000,7 +1192,7 @@
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>Sistem unghi mort Mercedes dedicat cu oglinzi dedicate GLC X253 2016-2022</t>
+          <t>Unghi mort Mercedes GLC X253 2016-2022 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr"/>
@@ -1015,6 +1207,16 @@
           <t>BSD-MB-03</t>
         </is>
       </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>GLC (X253) 2016-2022</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="40" customHeight="1">
       <c r="A21" s="6" t="inlineStr">
@@ -1024,7 +1226,7 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Sistem unghi mort Mercedes dedicat cu oglinzi dedicate GLB X247 2020-2024</t>
+          <t>Unghi mort Mercedes GLB X247 2020-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr"/>
@@ -1039,6 +1241,16 @@
           <t>BSD-MB-03</t>
         </is>
       </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>GLB (X247) 2020-2024</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="40" customHeight="1">
       <c r="A22" s="6" t="inlineStr">
@@ -1048,7 +1260,7 @@
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>Sistem unghi mort Mercedes dedicat cu oglinzi dedicate B-Class W247 2020-2024</t>
+          <t>Unghi mort Mercedes B-Class W247 2020-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr"/>
@@ -1063,6 +1275,16 @@
           <t>BSD-MB-03</t>
         </is>
       </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>B-Class (W247) 2020-2024</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="40" customHeight="1">
       <c r="A23" s="6" t="inlineStr">
@@ -1072,7 +1294,7 @@
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Sistem unghi mort Mercedes dedicat cu oglinzi dedicate EQC N293 2020-2024</t>
+          <t>Unghi mort Mercedes EQC N293 2020-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr"/>
@@ -1087,6 +1309,16 @@
           <t>BSD-MB-03</t>
         </is>
       </c>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>EQC (N293) 2020-2024</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="40" customHeight="1">
       <c r="A24" s="6" t="inlineStr">
@@ -1096,7 +1328,7 @@
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>Sistem unghi mort Mercedes dedicat cu oglinzi dedicate EQA H243 2022-2024</t>
+          <t>Unghi mort Mercedes EQA H243 2022-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr"/>
@@ -1111,6 +1343,16 @@
           <t>BSD-MB-03</t>
         </is>
       </c>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>EQA (H243) 2022-2024</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="40" customHeight="1">
       <c r="A25" s="6" t="inlineStr">
@@ -1120,7 +1362,7 @@
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Sistem unghi mort Mercedes dedicat cu oglinzi dedicate EQB X243 2022-2024</t>
+          <t>Unghi mort Mercedes EQB X243 2022-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr"/>
@@ -1135,6 +1377,16 @@
           <t>BSD-MB-03</t>
         </is>
       </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>EQB (X243) 2022-2024</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="40" customHeight="1">
       <c r="A26" s="6" t="inlineStr">
@@ -1144,7 +1396,7 @@
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>Sistem unghi mort Mercedes dedicat cu oglinzi dedicate S-Class W222 2014-2020</t>
+          <t>Unghi mort Mercedes S-Class W222 2014-2020 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr"/>
@@ -1159,6 +1411,16 @@
           <t>BSD-MB-03</t>
         </is>
       </c>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
+      <c r="H26" s="7" t="inlineStr">
+        <is>
+          <t>S-Class (W222) 2014-2020</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="40" customHeight="1">
       <c r="A27" s="6" t="inlineStr">
@@ -1168,7 +1430,7 @@
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>Sistem unghi mort Mercedes dedicat cu oglinzi dedicate CLS W257 2018-2023</t>
+          <t>Unghi mort Mercedes CLS W257 2018-2023 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr"/>
@@ -1183,6 +1445,16 @@
           <t>BSD-MB-03</t>
         </is>
       </c>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>CLS (W257) 2018-2023</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="40" customHeight="1">
       <c r="A28" s="6" t="inlineStr">
@@ -1192,7 +1464,7 @@
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>Sistem unghi mort Mercedes dedicat cu oglinzi dedicate GT AMG 2019-2023</t>
+          <t>Unghi mort Mercedes GT AMG 2019-2023 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr"/>
@@ -1207,6 +1479,16 @@
           <t>BSD-MB-03</t>
         </is>
       </c>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t>GT AMG 2019-2023</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="40" customHeight="1">
       <c r="A29" s="8" t="inlineStr">
@@ -1216,7 +1498,7 @@
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>Sistem unghi mort Mercedes dedicat cu oglinzi dedicate A-Class W177 2019-2024</t>
+          <t>Unghi mort Mercedes A-Class W177 2019-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
       <c r="C29" s="8" t="inlineStr"/>
@@ -1231,6 +1513,16 @@
           <t>BSD-MB-04</t>
         </is>
       </c>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
+      <c r="H29" s="9" t="inlineStr">
+        <is>
+          <t>A-Class (W177) 2019-2024</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="40" customHeight="1">
       <c r="A30" s="8" t="inlineStr">
@@ -1240,7 +1532,7 @@
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>Sistem unghi mort Mercedes dedicat cu oglinzi dedicate CLA W118 2020-2024</t>
+          <t>Unghi mort Mercedes CLA W118 2020-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
       <c r="C30" s="8" t="inlineStr"/>
@@ -1255,6 +1547,16 @@
           <t>BSD-MB-04</t>
         </is>
       </c>
+      <c r="G30" s="8" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
+      <c r="H30" s="9" t="inlineStr">
+        <is>
+          <t>CLA (W118) 2020-2024</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="40" customHeight="1">
       <c r="A31" s="10" t="inlineStr">
@@ -1264,7 +1566,7 @@
       </c>
       <c r="B31" s="11" t="inlineStr">
         <is>
-          <t>Sistem unghi mort Mercedes dedicat cu oglinzi dedicate Vito W447 2016-2024</t>
+          <t>Unghi mort Mercedes Vito W447 2016-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
       <c r="C31" s="10" t="inlineStr"/>
@@ -1279,6 +1581,16 @@
           <t>BSD-MB-05</t>
         </is>
       </c>
+      <c r="G31" s="10" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
+      <c r="H31" s="11" t="inlineStr">
+        <is>
+          <t>Vito (W447) 2016-2024</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="40" customHeight="1">
       <c r="A32" s="10" t="inlineStr">
@@ -1288,7 +1600,7 @@
       </c>
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>Sistem unghi mort Mercedes dedicat cu oglinzi dedicate V-Class W447 2016-2024</t>
+          <t>Unghi mort Mercedes V-Class W447 2016-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
       <c r="C32" s="10" t="inlineStr"/>
@@ -1303,6 +1615,16 @@
           <t>BSD-MB-05</t>
         </is>
       </c>
+      <c r="G32" s="10" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
+      <c r="H32" s="11" t="inlineStr">
+        <is>
+          <t>V-Class (W447) 2016-2024</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="40" customHeight="1">
       <c r="A33" s="10" t="inlineStr">
@@ -1312,7 +1634,7 @@
       </c>
       <c r="B33" s="11" t="inlineStr">
         <is>
-          <t>Sistem unghi mort Mercedes dedicat cu oglinzi dedicate EQV W447 2023-2024</t>
+          <t>Unghi mort Mercedes EQV W447 2023-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
       <c r="C33" s="10" t="inlineStr"/>
@@ -1327,6 +1649,16 @@
           <t>BSD-MB-05</t>
         </is>
       </c>
+      <c r="G33" s="10" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
+      <c r="H33" s="11" t="inlineStr">
+        <is>
+          <t>EQV (W447) 2023-2024</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="40" customHeight="1">
       <c r="A34" s="10" t="inlineStr">
@@ -1336,7 +1668,7 @@
       </c>
       <c r="B34" s="11" t="inlineStr">
         <is>
-          <t>Sistem unghi mort Mercedes dedicat cu oglinzi dedicate G-Class W463 2012+</t>
+          <t>Unghi mort Mercedes G-Class W463 2012+ - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
       <c r="C34" s="10" t="inlineStr"/>
@@ -1351,6 +1683,16 @@
           <t>BSD-MB-05</t>
         </is>
       </c>
+      <c r="G34" s="10" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
+      <c r="H34" s="11" t="inlineStr">
+        <is>
+          <t>G-Class (W463) 2012+</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="40" customHeight="1">
       <c r="A35" s="12" t="inlineStr">
@@ -1360,7 +1702,7 @@
       </c>
       <c r="B35" s="13" t="inlineStr">
         <is>
-          <t>Sistem unghi mort Mercedes dedicat cu oglinzi dedicate C-Class W206 2022-2024</t>
+          <t>Unghi mort Mercedes C-Class W206 2022-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
       <c r="C35" s="12" t="inlineStr"/>
@@ -1375,6 +1717,16 @@
           <t>BSD-MB-06</t>
         </is>
       </c>
+      <c r="G35" s="12" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
+      <c r="H35" s="13" t="inlineStr">
+        <is>
+          <t>C-Class (W206) 2022-2024</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="40" customHeight="1">
       <c r="A36" s="12" t="inlineStr">
@@ -1384,7 +1736,7 @@
       </c>
       <c r="B36" s="13" t="inlineStr">
         <is>
-          <t>Sistem unghi mort Mercedes dedicat cu oglinzi dedicate GLC X254 2023-2024</t>
+          <t>Unghi mort Mercedes GLC X254 2023-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
       <c r="C36" s="12" t="inlineStr"/>
@@ -1399,6 +1751,16 @@
           <t>BSD-MB-06</t>
         </is>
       </c>
+      <c r="G36" s="12" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
+      <c r="H36" s="13" t="inlineStr">
+        <is>
+          <t>GLC (X254) 2023-2024</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="40" customHeight="1">
       <c r="A37" s="12" t="inlineStr">
@@ -1408,7 +1770,7 @@
       </c>
       <c r="B37" s="13" t="inlineStr">
         <is>
-          <t>Sistem unghi mort Mercedes dedicat cu oglinzi dedicate EQS V297 2022-2024</t>
+          <t>Unghi mort Mercedes EQS V297 2022-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
       <c r="C37" s="12" t="inlineStr"/>
@@ -1423,6 +1785,16 @@
           <t>BSD-MB-06</t>
         </is>
       </c>
+      <c r="G37" s="12" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
+      <c r="H37" s="13" t="inlineStr">
+        <is>
+          <t>EQS (V297) 2022-2024</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="40" customHeight="1">
       <c r="A38" s="12" t="inlineStr">
@@ -1432,7 +1804,7 @@
       </c>
       <c r="B38" s="13" t="inlineStr">
         <is>
-          <t>Sistem unghi mort Mercedes dedicat cu oglinzi dedicate E-Class W214 2024</t>
+          <t>Unghi mort Mercedes E-Class W214 2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
       <c r="C38" s="12" t="inlineStr"/>
@@ -1447,6 +1819,16 @@
           <t>BSD-MB-06</t>
         </is>
       </c>
+      <c r="G38" s="12" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
+      <c r="H38" s="13" t="inlineStr">
+        <is>
+          <t>E-Class (W214) 2024</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="40" customHeight="1">
       <c r="A39" s="12" t="inlineStr">
@@ -1456,7 +1838,7 @@
       </c>
       <c r="B39" s="13" t="inlineStr">
         <is>
-          <t>Sistem unghi mort Mercedes dedicat cu oglinzi dedicate S-Class W223 2021-2024</t>
+          <t>Unghi mort Mercedes S-Class W223 2021-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
       <c r="C39" s="12" t="inlineStr"/>
@@ -1471,6 +1853,16 @@
           <t>BSD-MB-06</t>
         </is>
       </c>
+      <c r="G39" s="12" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
+      <c r="H39" s="13" t="inlineStr">
+        <is>
+          <t>S-Class (W223) 2021-2024</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="40" customHeight="1">
       <c r="A40" s="12" t="inlineStr">
@@ -1480,7 +1872,7 @@
       </c>
       <c r="B40" s="13" t="inlineStr">
         <is>
-          <t>Sistem unghi mort Mercedes dedicat cu oglinzi dedicate S Maybach W223 2021-2024</t>
+          <t>Unghi mort Mercedes S Maybach W223 2021-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
       <c r="C40" s="12" t="inlineStr"/>
@@ -1495,6 +1887,16 @@
           <t>BSD-MB-06</t>
         </is>
       </c>
+      <c r="G40" s="12" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
+      <c r="H40" s="13" t="inlineStr">
+        <is>
+          <t>S Maybach (W223) 2021-2024</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="40" customHeight="1">
       <c r="A41" s="12" t="inlineStr">
@@ -1504,7 +1906,7 @@
       </c>
       <c r="B41" s="13" t="inlineStr">
         <is>
-          <t>Sistem unghi mort Mercedes dedicat cu oglinzi dedicate CLE W236 2024</t>
+          <t>Unghi mort Mercedes CLE W236 2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
       <c r="C41" s="12" t="inlineStr"/>
@@ -1519,6 +1921,16 @@
           <t>BSD-MB-06</t>
         </is>
       </c>
+      <c r="G41" s="12" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
+      <c r="H41" s="13" t="inlineStr">
+        <is>
+          <t>CLE (W236) 2024</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="40" customHeight="1">
       <c r="A42" s="14" t="inlineStr">
@@ -1528,7 +1940,7 @@
       </c>
       <c r="B42" s="15" t="inlineStr">
         <is>
-          <t>Sistem unghi mort Mercedes dedicat cu oglinzi dedicate GLE W167 2020-2024</t>
+          <t>Unghi mort Mercedes GLE W167 2020-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
       <c r="C42" s="14" t="inlineStr"/>
@@ -1543,6 +1955,16 @@
           <t>BSD-MB-07</t>
         </is>
       </c>
+      <c r="G42" s="14" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
+      <c r="H42" s="15" t="inlineStr">
+        <is>
+          <t>GLE (W167) 2020-2024</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="40" customHeight="1">
       <c r="A43" s="14" t="inlineStr">
@@ -1552,7 +1974,7 @@
       </c>
       <c r="B43" s="15" t="inlineStr">
         <is>
-          <t>Sistem unghi mort Mercedes dedicat cu oglinzi dedicate GLS X167 2020-2024</t>
+          <t>Unghi mort Mercedes GLS X167 2020-2024 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
       <c r="C43" s="14" t="inlineStr"/>
@@ -1567,6 +1989,16 @@
           <t>BSD-MB-07</t>
         </is>
       </c>
+      <c r="G43" s="14" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
+      <c r="H43" s="15" t="inlineStr">
+        <is>
+          <t>GLS (X167) 2020-2024</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="40" customHeight="1">
       <c r="A44" s="14" t="inlineStr">
@@ -1576,7 +2008,7 @@
       </c>
       <c r="B44" s="15" t="inlineStr">
         <is>
-          <t>Sistem unghi mort Mercedes dedicat cu oglinzi dedicate G-Class W463 2019-2022</t>
+          <t>Unghi mort Mercedes G-Class W463 2019-2022 - Sistem BSD dedicat cu oglinzi</t>
         </is>
       </c>
       <c r="C44" s="14" t="inlineStr"/>
@@ -1589,6 +2021,16 @@
       <c r="F44" s="14" t="inlineStr">
         <is>
           <t>BSD-MB-07</t>
+        </is>
+      </c>
+      <c r="G44" s="14" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
+      <c r="H44" s="15" t="inlineStr">
+        <is>
+          <t>G-Class (W463) 2019-2022</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
BSD Mercedes - atribute complete din feed vehicule
</commit_message>
<xml_diff>
--- a/BSD-Mercedes-Benz-Final.xlsx
+++ b/BSD-Mercedes-Benz-Final.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sistem BSD Mercedes-Benz" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="BSD Mercedes-Benz" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -517,17 +517,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H44"/>
+  <dimension ref="A1:K44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="70" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="68" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="35" customHeight="1">
@@ -563,16 +566,31 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Marca (Atribut)</t>
+          <t>Marca</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Model (Atribut)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="40" customHeight="1">
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Cod Caroserie</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>An Start</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>An Stop</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="38" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>BSD-01+BSD-MB-01-V1</t>
@@ -580,7 +598,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes C-Class W204 2009-2014 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Unghi mort Mercedes C-Class W204 2009-2014 - Sistem BSD cu oglinzi dedicate</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr"/>
@@ -600,13 +618,24 @@
           <t>Mercedes-Benz</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>C-Class (W204) 2009-2014</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="40" customHeight="1">
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>C-Class</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>W204</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="n">
+        <v>2007</v>
+      </c>
+      <c r="K2" s="2" t="n">
+        <v>2014</v>
+      </c>
+    </row>
+    <row r="3" ht="38" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>BSD-01+BSD-MB-01-V2</t>
@@ -614,7 +643,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes E-Class W212 2010-2015 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Unghi mort Mercedes E-Class W212 2010-2015 - Sistem BSD cu oglinzi dedicate</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr"/>
@@ -634,13 +663,24 @@
           <t>Mercedes-Benz</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>E-Class (W212) 2010-2015</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="40" customHeight="1">
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>E-Class</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>W212</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>2009</v>
+      </c>
+      <c r="K3" s="2" t="n">
+        <v>2016</v>
+      </c>
+    </row>
+    <row r="4" ht="38" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>BSD-01+BSD-MB-01-V3</t>
@@ -648,7 +688,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes GLK W204 2009-2015 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Unghi mort Mercedes GLK W204 2009-2015 - Sistem BSD cu oglinzi dedicate</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr"/>
@@ -668,13 +708,24 @@
           <t>Mercedes-Benz</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>GLK (W204) 2009-2015</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="40" customHeight="1">
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>GLK</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>X204</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="n">
+        <v>2008</v>
+      </c>
+      <c r="K4" s="2" t="n">
+        <v>2015</v>
+      </c>
+    </row>
+    <row r="5" ht="38" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>BSD-01+BSD-MB-01-V4</t>
@@ -682,7 +733,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes GLA X156 2015-2019 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Unghi mort Mercedes GLA X156 2015-2019 - Sistem BSD cu oglinzi dedicate</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr"/>
@@ -702,13 +753,24 @@
           <t>Mercedes-Benz</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>GLA (X156) 2015-2019</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="40" customHeight="1">
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>GLA</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>X156</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="n">
+        <v>2013</v>
+      </c>
+      <c r="K5" s="2" t="n">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="6" ht="38" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>BSD-01+BSD-MB-01-V5</t>
@@ -716,7 +778,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes A-Class W176 2013-2018 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Unghi mort Mercedes A-Class W176 2013-2018 - Sistem BSD cu oglinzi dedicate</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr"/>
@@ -736,13 +798,24 @@
           <t>Mercedes-Benz</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>A-Class (W176) 2013-2018</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="40" customHeight="1">
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>A-Class</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>W176</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v>2012</v>
+      </c>
+      <c r="K6" s="2" t="n">
+        <v>2018</v>
+      </c>
+    </row>
+    <row r="7" ht="38" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>BSD-01+BSD-MB-01-V6</t>
@@ -750,7 +823,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes B-Class W246 2012-2019 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Unghi mort Mercedes B-Class W246 2012-2019 - Sistem BSD cu oglinzi dedicate</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr"/>
@@ -770,13 +843,24 @@
           <t>Mercedes-Benz</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
-        <is>
-          <t>B-Class (W246) 2012-2019</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="40" customHeight="1">
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>B-Class</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>W246</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="n">
+        <v>2011</v>
+      </c>
+      <c r="K7" s="2" t="n">
+        <v>2018</v>
+      </c>
+    </row>
+    <row r="8" ht="38" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>BSD-01+BSD-MB-01-V7</t>
@@ -784,7 +868,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes CLA W117 2014-2019 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Unghi mort Mercedes CLA W117 2014-2019 - Sistem BSD cu oglinzi dedicate</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr"/>
@@ -804,13 +888,24 @@
           <t>Mercedes-Benz</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>CLA (W117) 2014-2019</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="40" customHeight="1">
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>CLA</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>C117</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="n">
+        <v>2013</v>
+      </c>
+      <c r="K8" s="2" t="n">
+        <v>2019</v>
+      </c>
+    </row>
+    <row r="9" ht="38" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>BSD-01+BSD-MB-01-V8</t>
@@ -818,7 +913,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes S-Class W221 2010-2013 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Unghi mort Mercedes S-Class W221 2010-2013 - Sistem BSD cu oglinzi dedicate</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr"/>
@@ -838,13 +933,24 @@
           <t>Mercedes-Benz</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr">
-        <is>
-          <t>S-Class (W221) 2010-2013</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="40" customHeight="1">
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>S-Class</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>W221</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="n">
+        <v>2005</v>
+      </c>
+      <c r="K9" s="2" t="n">
+        <v>2013</v>
+      </c>
+    </row>
+    <row r="10" ht="38" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>BSD-01+BSD-MB-01-V9</t>
@@ -852,7 +958,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes CLS W218 2011-2017 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Unghi mort Mercedes CLS W218 2011-2017 - Sistem BSD cu oglinzi dedicate</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr"/>
@@ -872,13 +978,24 @@
           <t>Mercedes-Benz</t>
         </is>
       </c>
-      <c r="H10" s="3" t="inlineStr">
-        <is>
-          <t>CLS (W218) 2011-2017</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="40" customHeight="1">
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>CLS</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>C218</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="n">
+        <v>2011</v>
+      </c>
+      <c r="K10" s="2" t="n">
+        <v>2018</v>
+      </c>
+    </row>
+    <row r="11" ht="38" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>BSD-01+BSD-MB-02-V1</t>
@@ -886,7 +1003,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes ML W164 2010-2015 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Unghi mort Mercedes ML W164 2010-2015 - Sistem BSD cu oglinzi dedicate</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr"/>
@@ -906,13 +1023,24 @@
           <t>Mercedes-Benz</t>
         </is>
       </c>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>ML (W164) 2010-2015</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="40" customHeight="1">
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>W164</t>
+        </is>
+      </c>
+      <c r="J11" s="4" t="n">
+        <v>2005</v>
+      </c>
+      <c r="K11" s="4" t="n">
+        <v>2011</v>
+      </c>
+    </row>
+    <row r="12" ht="38" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
           <t>BSD-01+BSD-MB-02-V2</t>
@@ -920,7 +1048,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes GLE W166 2015-2019 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Unghi mort Mercedes GLE W166 2015-2019 - Sistem BSD cu oglinzi dedicate</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr"/>
@@ -940,13 +1068,24 @@
           <t>Mercedes-Benz</t>
         </is>
       </c>
-      <c r="H12" s="5" t="inlineStr">
-        <is>
-          <t>GLE (W166) 2015-2019</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="40" customHeight="1">
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>GLE</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>W166</t>
+        </is>
+      </c>
+      <c r="J12" s="4" t="n">
+        <v>2015</v>
+      </c>
+      <c r="K12" s="4" t="n">
+        <v>2018</v>
+      </c>
+    </row>
+    <row r="13" ht="38" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
           <t>BSD-01+BSD-MB-02-V3</t>
@@ -954,7 +1093,7 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes GLS X166 2016-2019 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Unghi mort Mercedes GLS X166 2016-2019 - Sistem BSD cu oglinzi dedicate</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr"/>
@@ -974,13 +1113,24 @@
           <t>Mercedes-Benz</t>
         </is>
       </c>
-      <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>GLS (X166) 2016-2019</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="40" customHeight="1">
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>GLS</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>X166</t>
+        </is>
+      </c>
+      <c r="J13" s="4" t="n">
+        <v>2015</v>
+      </c>
+      <c r="K13" s="4" t="n">
+        <v>2019</v>
+      </c>
+    </row>
+    <row r="14" ht="38" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
           <t>BSD-01+BSD-MB-02-V4</t>
@@ -988,7 +1138,7 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes GL X166 2013-2016 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Unghi mort Mercedes GL X166 2013-2016 - Sistem BSD cu oglinzi dedicate</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr"/>
@@ -1008,13 +1158,24 @@
           <t>Mercedes-Benz</t>
         </is>
       </c>
-      <c r="H14" s="5" t="inlineStr">
-        <is>
-          <t>GL (X166) 2013-2016</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="40" customHeight="1">
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>GL</t>
+        </is>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>X166</t>
+        </is>
+      </c>
+      <c r="J14" s="4" t="n">
+        <v>2012</v>
+      </c>
+      <c r="K14" s="4" t="n">
+        <v>2016</v>
+      </c>
+    </row>
+    <row r="15" ht="38" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
           <t>BSD-01+BSD-MB-02-V5</t>
@@ -1022,7 +1183,7 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes R-Class W251 2009-2017 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Unghi mort Mercedes R-Class W251 2009-2017 - Sistem BSD cu oglinzi dedicate</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr"/>
@@ -1042,13 +1203,24 @@
           <t>Mercedes-Benz</t>
         </is>
       </c>
-      <c r="H15" s="5" t="inlineStr">
-        <is>
-          <t>R-Class (W251) 2009-2017</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="40" customHeight="1">
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>R-Class</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>W251</t>
+        </is>
+      </c>
+      <c r="J15" s="4" t="n">
+        <v>2005</v>
+      </c>
+      <c r="K15" s="4" t="n">
+        <v>2017</v>
+      </c>
+    </row>
+    <row r="16" ht="38" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
           <t>BSD-01+BSD-MB-02-V6</t>
@@ -1056,7 +1228,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes G-Class W463 2013-2018 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Unghi mort Mercedes G-Class W463 2013-2018 - Sistem BSD cu oglinzi dedicate</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr"/>
@@ -1076,13 +1248,24 @@
           <t>Mercedes-Benz</t>
         </is>
       </c>
-      <c r="H16" s="5" t="inlineStr">
-        <is>
-          <t>G-Class (W463) 2013-2018</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="40" customHeight="1">
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>G-Class</t>
+        </is>
+      </c>
+      <c r="I16" s="4" t="inlineStr">
+        <is>
+          <t>W463</t>
+        </is>
+      </c>
+      <c r="J16" s="4" t="n">
+        <v>2008</v>
+      </c>
+      <c r="K16" s="4" t="n">
+        <v>2018</v>
+      </c>
+    </row>
+    <row r="17" ht="38" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
         <is>
           <t>BSD-01+BSD-MB-03-V1</t>
@@ -1090,7 +1273,7 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes C-Class W205 2015-2021 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Unghi mort Mercedes C-Class W205 2015-2021 - Sistem BSD cu oglinzi dedicate</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr"/>
@@ -1110,13 +1293,24 @@
           <t>Mercedes-Benz</t>
         </is>
       </c>
-      <c r="H17" s="7" t="inlineStr">
-        <is>
-          <t>C-Class (W205) 2015-2021</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="40" customHeight="1">
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>C-Class</t>
+        </is>
+      </c>
+      <c r="I17" s="6" t="inlineStr">
+        <is>
+          <t>W205</t>
+        </is>
+      </c>
+      <c r="J17" s="6" t="n">
+        <v>2014</v>
+      </c>
+      <c r="K17" s="6" t="n">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="18" ht="38" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
         <is>
           <t>BSD-01+BSD-MB-03-V2</t>
@@ -1124,7 +1318,7 @@
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes E-Class W213 2016-2023 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Unghi mort Mercedes E-Class W213 2016-2023 - Sistem BSD cu oglinzi dedicate</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr"/>
@@ -1144,13 +1338,24 @@
           <t>Mercedes-Benz</t>
         </is>
       </c>
-      <c r="H18" s="7" t="inlineStr">
-        <is>
-          <t>E-Class (W213) 2016-2023</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="40" customHeight="1">
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>E-Class</t>
+        </is>
+      </c>
+      <c r="I18" s="6" t="inlineStr">
+        <is>
+          <t>W213</t>
+        </is>
+      </c>
+      <c r="J18" s="6" t="n">
+        <v>2016</v>
+      </c>
+      <c r="K18" s="6" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="19" ht="38" customHeight="1">
       <c r="A19" s="6" t="inlineStr">
         <is>
           <t>BSD-01+BSD-MB-03-V3</t>
@@ -1158,7 +1363,7 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes GLA H247 2020-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Unghi mort Mercedes GLA H247 2020-2024 - Sistem BSD cu oglinzi dedicate</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr"/>
@@ -1178,13 +1383,24 @@
           <t>Mercedes-Benz</t>
         </is>
       </c>
-      <c r="H19" s="7" t="inlineStr">
-        <is>
-          <t>GLA (H247) 2020-2024</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="40" customHeight="1">
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>GLA</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="inlineStr">
+        <is>
+          <t>H247</t>
+        </is>
+      </c>
+      <c r="J19" s="6" t="n">
+        <v>2020</v>
+      </c>
+      <c r="K19" s="6" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="20" ht="38" customHeight="1">
       <c r="A20" s="6" t="inlineStr">
         <is>
           <t>BSD-01+BSD-MB-03-V4</t>
@@ -1192,7 +1408,7 @@
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes GLC X253 2016-2022 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Unghi mort Mercedes GLC X253 2016-2022 - Sistem BSD cu oglinzi dedicate</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr"/>
@@ -1212,13 +1428,24 @@
           <t>Mercedes-Benz</t>
         </is>
       </c>
-      <c r="H20" s="7" t="inlineStr">
-        <is>
-          <t>GLC (X253) 2016-2022</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="40" customHeight="1">
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>GLC</t>
+        </is>
+      </c>
+      <c r="I20" s="6" t="inlineStr">
+        <is>
+          <t>X253</t>
+        </is>
+      </c>
+      <c r="J20" s="6" t="n">
+        <v>2015</v>
+      </c>
+      <c r="K20" s="6" t="n">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="21" ht="38" customHeight="1">
       <c r="A21" s="6" t="inlineStr">
         <is>
           <t>BSD-01+BSD-MB-03-V5</t>
@@ -1226,7 +1453,7 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes GLB X247 2020-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Unghi mort Mercedes GLB X247 2020-2024 - Sistem BSD cu oglinzi dedicate</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr"/>
@@ -1246,13 +1473,24 @@
           <t>Mercedes-Benz</t>
         </is>
       </c>
-      <c r="H21" s="7" t="inlineStr">
-        <is>
-          <t>GLB (X247) 2020-2024</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="40" customHeight="1">
+      <c r="H21" s="6" t="inlineStr">
+        <is>
+          <t>GLB</t>
+        </is>
+      </c>
+      <c r="I21" s="6" t="inlineStr">
+        <is>
+          <t>X247</t>
+        </is>
+      </c>
+      <c r="J21" s="6" t="n">
+        <v>2019</v>
+      </c>
+      <c r="K21" s="6" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="22" ht="38" customHeight="1">
       <c r="A22" s="6" t="inlineStr">
         <is>
           <t>BSD-01+BSD-MB-03-V6</t>
@@ -1260,7 +1498,7 @@
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes B-Class W247 2020-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Unghi mort Mercedes B-Class W247 2020-2024 - Sistem BSD cu oglinzi dedicate</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr"/>
@@ -1280,13 +1518,24 @@
           <t>Mercedes-Benz</t>
         </is>
       </c>
-      <c r="H22" s="7" t="inlineStr">
-        <is>
-          <t>B-Class (W247) 2020-2024</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="40" customHeight="1">
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>B-Class</t>
+        </is>
+      </c>
+      <c r="I22" s="6" t="inlineStr">
+        <is>
+          <t>W247</t>
+        </is>
+      </c>
+      <c r="J22" s="6" t="n">
+        <v>2018</v>
+      </c>
+      <c r="K22" s="6" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="23" ht="38" customHeight="1">
       <c r="A23" s="6" t="inlineStr">
         <is>
           <t>BSD-01+BSD-MB-03-V7</t>
@@ -1294,7 +1543,7 @@
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes EQC N293 2020-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Unghi mort Mercedes EQC N293 2020-2024 - Sistem BSD cu oglinzi dedicate</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr"/>
@@ -1314,13 +1563,24 @@
           <t>Mercedes-Benz</t>
         </is>
       </c>
-      <c r="H23" s="7" t="inlineStr">
-        <is>
-          <t>EQC (N293) 2020-2024</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="40" customHeight="1">
+      <c r="H23" s="6" t="inlineStr">
+        <is>
+          <t>EQC</t>
+        </is>
+      </c>
+      <c r="I23" s="6" t="inlineStr">
+        <is>
+          <t>N293</t>
+        </is>
+      </c>
+      <c r="J23" s="6" t="n">
+        <v>2019</v>
+      </c>
+      <c r="K23" s="6" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="24" ht="38" customHeight="1">
       <c r="A24" s="6" t="inlineStr">
         <is>
           <t>BSD-01+BSD-MB-03-V8</t>
@@ -1328,7 +1588,7 @@
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes EQA H243 2022-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Unghi mort Mercedes EQA H243 2022-2024 - Sistem BSD cu oglinzi dedicate</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr"/>
@@ -1348,13 +1608,24 @@
           <t>Mercedes-Benz</t>
         </is>
       </c>
-      <c r="H24" s="7" t="inlineStr">
-        <is>
-          <t>EQA (H243) 2022-2024</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="40" customHeight="1">
+      <c r="H24" s="6" t="inlineStr">
+        <is>
+          <t>EQA</t>
+        </is>
+      </c>
+      <c r="I24" s="6" t="inlineStr">
+        <is>
+          <t>H243</t>
+        </is>
+      </c>
+      <c r="J24" s="6" t="n">
+        <v>2021</v>
+      </c>
+      <c r="K24" s="6" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="25" ht="38" customHeight="1">
       <c r="A25" s="6" t="inlineStr">
         <is>
           <t>BSD-01+BSD-MB-03-V9</t>
@@ -1362,7 +1633,7 @@
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes EQB X243 2022-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Unghi mort Mercedes EQB X243 2022-2024 - Sistem BSD cu oglinzi dedicate</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr"/>
@@ -1382,13 +1653,24 @@
           <t>Mercedes-Benz</t>
         </is>
       </c>
-      <c r="H25" s="7" t="inlineStr">
-        <is>
-          <t>EQB (X243) 2022-2024</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="40" customHeight="1">
+      <c r="H25" s="6" t="inlineStr">
+        <is>
+          <t>EQB</t>
+        </is>
+      </c>
+      <c r="I25" s="6" t="inlineStr">
+        <is>
+          <t>X243</t>
+        </is>
+      </c>
+      <c r="J25" s="6" t="n">
+        <v>2021</v>
+      </c>
+      <c r="K25" s="6" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="26" ht="38" customHeight="1">
       <c r="A26" s="6" t="inlineStr">
         <is>
           <t>BSD-01+BSD-MB-03-V10</t>
@@ -1396,7 +1678,7 @@
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes S-Class W222 2014-2020 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Unghi mort Mercedes S-Class W222 2014-2020 - Sistem BSD cu oglinzi dedicate</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr"/>
@@ -1416,13 +1698,24 @@
           <t>Mercedes-Benz</t>
         </is>
       </c>
-      <c r="H26" s="7" t="inlineStr">
-        <is>
-          <t>S-Class (W222) 2014-2020</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="40" customHeight="1">
+      <c r="H26" s="6" t="inlineStr">
+        <is>
+          <t>S-Class</t>
+        </is>
+      </c>
+      <c r="I26" s="6" t="inlineStr">
+        <is>
+          <t>W222</t>
+        </is>
+      </c>
+      <c r="J26" s="6" t="n">
+        <v>2013</v>
+      </c>
+      <c r="K26" s="6" t="n">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="27" ht="38" customHeight="1">
       <c r="A27" s="6" t="inlineStr">
         <is>
           <t>BSD-01+BSD-MB-03-V11</t>
@@ -1430,7 +1723,7 @@
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes CLS W257 2018-2023 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Unghi mort Mercedes CLS W257 2018-2023 - Sistem BSD cu oglinzi dedicate</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr"/>
@@ -1450,13 +1743,24 @@
           <t>Mercedes-Benz</t>
         </is>
       </c>
-      <c r="H27" s="7" t="inlineStr">
-        <is>
-          <t>CLS (W257) 2018-2023</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="40" customHeight="1">
+      <c r="H27" s="6" t="inlineStr">
+        <is>
+          <t>CLS</t>
+        </is>
+      </c>
+      <c r="I27" s="6" t="inlineStr">
+        <is>
+          <t>C257</t>
+        </is>
+      </c>
+      <c r="J27" s="6" t="n">
+        <v>2018</v>
+      </c>
+      <c r="K27" s="6" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="28" ht="38" customHeight="1">
       <c r="A28" s="6" t="inlineStr">
         <is>
           <t>BSD-01+BSD-MB-03-V12</t>
@@ -1464,7 +1768,7 @@
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes GT AMG 2019-2023 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Unghi mort Mercedes GT AMG 2019-2023 - Sistem BSD cu oglinzi dedicate</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr"/>
@@ -1484,13 +1788,24 @@
           <t>Mercedes-Benz</t>
         </is>
       </c>
-      <c r="H28" s="7" t="inlineStr">
-        <is>
-          <t>GT AMG 2019-2023</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="40" customHeight="1">
+      <c r="H28" s="6" t="inlineStr">
+        <is>
+          <t>GT AMG</t>
+        </is>
+      </c>
+      <c r="I28" s="6" t="inlineStr">
+        <is>
+          <t>C190</t>
+        </is>
+      </c>
+      <c r="J28" s="6" t="n">
+        <v>2014</v>
+      </c>
+      <c r="K28" s="6" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="29" ht="38" customHeight="1">
       <c r="A29" s="8" t="inlineStr">
         <is>
           <t>BSD-01+BSD-MB-04-V1</t>
@@ -1498,7 +1813,7 @@
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes A-Class W177 2019-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Unghi mort Mercedes A-Class W177 2019-2024 - Sistem BSD cu oglinzi dedicate</t>
         </is>
       </c>
       <c r="C29" s="8" t="inlineStr"/>
@@ -1518,13 +1833,24 @@
           <t>Mercedes-Benz</t>
         </is>
       </c>
-      <c r="H29" s="9" t="inlineStr">
-        <is>
-          <t>A-Class (W177) 2019-2024</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="40" customHeight="1">
+      <c r="H29" s="8" t="inlineStr">
+        <is>
+          <t>A-Class</t>
+        </is>
+      </c>
+      <c r="I29" s="8" t="inlineStr">
+        <is>
+          <t>W177</t>
+        </is>
+      </c>
+      <c r="J29" s="8" t="n">
+        <v>2018</v>
+      </c>
+      <c r="K29" s="8" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="30" ht="38" customHeight="1">
       <c r="A30" s="8" t="inlineStr">
         <is>
           <t>BSD-01+BSD-MB-04-V2</t>
@@ -1532,7 +1858,7 @@
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes CLA W118 2020-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Unghi mort Mercedes CLA W118 2020-2024 - Sistem BSD cu oglinzi dedicate</t>
         </is>
       </c>
       <c r="C30" s="8" t="inlineStr"/>
@@ -1552,13 +1878,24 @@
           <t>Mercedes-Benz</t>
         </is>
       </c>
-      <c r="H30" s="9" t="inlineStr">
-        <is>
-          <t>CLA (W118) 2020-2024</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="40" customHeight="1">
+      <c r="H30" s="8" t="inlineStr">
+        <is>
+          <t>CLA</t>
+        </is>
+      </c>
+      <c r="I30" s="8" t="inlineStr">
+        <is>
+          <t>C118</t>
+        </is>
+      </c>
+      <c r="J30" s="8" t="n">
+        <v>2019</v>
+      </c>
+      <c r="K30" s="8" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="31" ht="38" customHeight="1">
       <c r="A31" s="10" t="inlineStr">
         <is>
           <t>BSD-01+BSD-MB-05-V1</t>
@@ -1566,7 +1903,7 @@
       </c>
       <c r="B31" s="11" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes Vito W447 2016-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Unghi mort Mercedes Vito W447 2016-2024 - Sistem BSD cu oglinzi dedicate</t>
         </is>
       </c>
       <c r="C31" s="10" t="inlineStr"/>
@@ -1586,13 +1923,24 @@
           <t>Mercedes-Benz</t>
         </is>
       </c>
-      <c r="H31" s="11" t="inlineStr">
-        <is>
-          <t>Vito (W447) 2016-2024</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="40" customHeight="1">
+      <c r="H31" s="10" t="inlineStr">
+        <is>
+          <t>Vito</t>
+        </is>
+      </c>
+      <c r="I31" s="10" t="inlineStr">
+        <is>
+          <t>W447</t>
+        </is>
+      </c>
+      <c r="J31" s="10" t="n">
+        <v>2014</v>
+      </c>
+      <c r="K31" s="10" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="32" ht="38" customHeight="1">
       <c r="A32" s="10" t="inlineStr">
         <is>
           <t>BSD-01+BSD-MB-05-V2</t>
@@ -1600,7 +1948,7 @@
       </c>
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes V-Class W447 2016-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Unghi mort Mercedes V-Class W447 2016-2024 - Sistem BSD cu oglinzi dedicate</t>
         </is>
       </c>
       <c r="C32" s="10" t="inlineStr"/>
@@ -1620,13 +1968,24 @@
           <t>Mercedes-Benz</t>
         </is>
       </c>
-      <c r="H32" s="11" t="inlineStr">
-        <is>
-          <t>V-Class (W447) 2016-2024</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="40" customHeight="1">
+      <c r="H32" s="10" t="inlineStr">
+        <is>
+          <t>V-Class</t>
+        </is>
+      </c>
+      <c r="I32" s="10" t="inlineStr">
+        <is>
+          <t>W447</t>
+        </is>
+      </c>
+      <c r="J32" s="10" t="n">
+        <v>2014</v>
+      </c>
+      <c r="K32" s="10" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="33" ht="38" customHeight="1">
       <c r="A33" s="10" t="inlineStr">
         <is>
           <t>BSD-01+BSD-MB-05-V3</t>
@@ -1634,7 +1993,7 @@
       </c>
       <c r="B33" s="11" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes EQV W447 2023-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Unghi mort Mercedes EQV W447 2023-2024 - Sistem BSD cu oglinzi dedicate</t>
         </is>
       </c>
       <c r="C33" s="10" t="inlineStr"/>
@@ -1654,13 +2013,24 @@
           <t>Mercedes-Benz</t>
         </is>
       </c>
-      <c r="H33" s="11" t="inlineStr">
-        <is>
-          <t>EQV (W447) 2023-2024</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="40" customHeight="1">
+      <c r="H33" s="10" t="inlineStr">
+        <is>
+          <t>EQV</t>
+        </is>
+      </c>
+      <c r="I33" s="10" t="inlineStr">
+        <is>
+          <t>W447</t>
+        </is>
+      </c>
+      <c r="J33" s="10" t="n">
+        <v>2020</v>
+      </c>
+      <c r="K33" s="10" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="34" ht="38" customHeight="1">
       <c r="A34" s="10" t="inlineStr">
         <is>
           <t>BSD-01+BSD-MB-05-V4</t>
@@ -1668,7 +2038,7 @@
       </c>
       <c r="B34" s="11" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes G-Class W463 2012+ - Sistem BSD dedicat cu oglinzi</t>
+          <t>Unghi mort Mercedes G-Class W463 2012+ - Sistem BSD cu oglinzi dedicate</t>
         </is>
       </c>
       <c r="C34" s="10" t="inlineStr"/>
@@ -1688,13 +2058,24 @@
           <t>Mercedes-Benz</t>
         </is>
       </c>
-      <c r="H34" s="11" t="inlineStr">
-        <is>
-          <t>G-Class (W463) 2012+</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="40" customHeight="1">
+      <c r="H34" s="10" t="inlineStr">
+        <is>
+          <t>G-Class</t>
+        </is>
+      </c>
+      <c r="I34" s="10" t="inlineStr">
+        <is>
+          <t>W463</t>
+        </is>
+      </c>
+      <c r="J34" s="10" t="n">
+        <v>2012</v>
+      </c>
+      <c r="K34" s="10" t="n">
+        <v>2018</v>
+      </c>
+    </row>
+    <row r="35" ht="38" customHeight="1">
       <c r="A35" s="12" t="inlineStr">
         <is>
           <t>BSD-01+BSD-MB-06-V1</t>
@@ -1702,7 +2083,7 @@
       </c>
       <c r="B35" s="13" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes C-Class W206 2022-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Unghi mort Mercedes C-Class W206 2022-2024 - Sistem BSD cu oglinzi dedicate</t>
         </is>
       </c>
       <c r="C35" s="12" t="inlineStr"/>
@@ -1722,13 +2103,24 @@
           <t>Mercedes-Benz</t>
         </is>
       </c>
-      <c r="H35" s="13" t="inlineStr">
-        <is>
-          <t>C-Class (W206) 2022-2024</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="40" customHeight="1">
+      <c r="H35" s="12" t="inlineStr">
+        <is>
+          <t>C-Class</t>
+        </is>
+      </c>
+      <c r="I35" s="12" t="inlineStr">
+        <is>
+          <t>W206</t>
+        </is>
+      </c>
+      <c r="J35" s="12" t="n">
+        <v>2021</v>
+      </c>
+      <c r="K35" s="12" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="36" ht="38" customHeight="1">
       <c r="A36" s="12" t="inlineStr">
         <is>
           <t>BSD-01+BSD-MB-06-V2</t>
@@ -1736,7 +2128,7 @@
       </c>
       <c r="B36" s="13" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes GLC X254 2023-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Unghi mort Mercedes GLC X254 2023-2024 - Sistem BSD cu oglinzi dedicate</t>
         </is>
       </c>
       <c r="C36" s="12" t="inlineStr"/>
@@ -1756,13 +2148,24 @@
           <t>Mercedes-Benz</t>
         </is>
       </c>
-      <c r="H36" s="13" t="inlineStr">
-        <is>
-          <t>GLC (X254) 2023-2024</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="40" customHeight="1">
+      <c r="H36" s="12" t="inlineStr">
+        <is>
+          <t>GLC</t>
+        </is>
+      </c>
+      <c r="I36" s="12" t="inlineStr">
+        <is>
+          <t>X254</t>
+        </is>
+      </c>
+      <c r="J36" s="12" t="n">
+        <v>2022</v>
+      </c>
+      <c r="K36" s="12" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="37" ht="38" customHeight="1">
       <c r="A37" s="12" t="inlineStr">
         <is>
           <t>BSD-01+BSD-MB-06-V3</t>
@@ -1770,7 +2173,7 @@
       </c>
       <c r="B37" s="13" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes EQS V297 2022-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Unghi mort Mercedes EQS V297 2022-2024 - Sistem BSD cu oglinzi dedicate</t>
         </is>
       </c>
       <c r="C37" s="12" t="inlineStr"/>
@@ -1790,13 +2193,24 @@
           <t>Mercedes-Benz</t>
         </is>
       </c>
-      <c r="H37" s="13" t="inlineStr">
-        <is>
-          <t>EQS (V297) 2022-2024</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="40" customHeight="1">
+      <c r="H37" s="12" t="inlineStr">
+        <is>
+          <t>EQS</t>
+        </is>
+      </c>
+      <c r="I37" s="12" t="inlineStr">
+        <is>
+          <t>V297</t>
+        </is>
+      </c>
+      <c r="J37" s="12" t="n">
+        <v>2021</v>
+      </c>
+      <c r="K37" s="12" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="38" ht="38" customHeight="1">
       <c r="A38" s="12" t="inlineStr">
         <is>
           <t>BSD-01+BSD-MB-06-V4</t>
@@ -1804,7 +2218,7 @@
       </c>
       <c r="B38" s="13" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes E-Class W214 2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Unghi mort Mercedes E-Class W214 2024 - Sistem BSD cu oglinzi dedicate</t>
         </is>
       </c>
       <c r="C38" s="12" t="inlineStr"/>
@@ -1824,13 +2238,24 @@
           <t>Mercedes-Benz</t>
         </is>
       </c>
-      <c r="H38" s="13" t="inlineStr">
-        <is>
-          <t>E-Class (W214) 2024</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="40" customHeight="1">
+      <c r="H38" s="12" t="inlineStr">
+        <is>
+          <t>E-Class</t>
+        </is>
+      </c>
+      <c r="I38" s="12" t="inlineStr">
+        <is>
+          <t>W214</t>
+        </is>
+      </c>
+      <c r="J38" s="12" t="n">
+        <v>2023</v>
+      </c>
+      <c r="K38" s="12" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="39" ht="38" customHeight="1">
       <c r="A39" s="12" t="inlineStr">
         <is>
           <t>BSD-01+BSD-MB-06-V5</t>
@@ -1838,7 +2263,7 @@
       </c>
       <c r="B39" s="13" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes S-Class W223 2021-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Unghi mort Mercedes S-Class W223 2021-2024 - Sistem BSD cu oglinzi dedicate</t>
         </is>
       </c>
       <c r="C39" s="12" t="inlineStr"/>
@@ -1858,13 +2283,24 @@
           <t>Mercedes-Benz</t>
         </is>
       </c>
-      <c r="H39" s="13" t="inlineStr">
-        <is>
-          <t>S-Class (W223) 2021-2024</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="40" customHeight="1">
+      <c r="H39" s="12" t="inlineStr">
+        <is>
+          <t>S-Class</t>
+        </is>
+      </c>
+      <c r="I39" s="12" t="inlineStr">
+        <is>
+          <t>W223</t>
+        </is>
+      </c>
+      <c r="J39" s="12" t="n">
+        <v>2020</v>
+      </c>
+      <c r="K39" s="12" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="40" ht="38" customHeight="1">
       <c r="A40" s="12" t="inlineStr">
         <is>
           <t>BSD-01+BSD-MB-06-V6</t>
@@ -1872,7 +2308,7 @@
       </c>
       <c r="B40" s="13" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes S Maybach W223 2021-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Unghi mort Mercedes S Maybach W223 2021-2024 - Sistem BSD cu oglinzi dedicate</t>
         </is>
       </c>
       <c r="C40" s="12" t="inlineStr"/>
@@ -1892,13 +2328,24 @@
           <t>Mercedes-Benz</t>
         </is>
       </c>
-      <c r="H40" s="13" t="inlineStr">
-        <is>
-          <t>S Maybach (W223) 2021-2024</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="40" customHeight="1">
+      <c r="H40" s="12" t="inlineStr">
+        <is>
+          <t>S Maybach</t>
+        </is>
+      </c>
+      <c r="I40" s="12" t="inlineStr">
+        <is>
+          <t>W223</t>
+        </is>
+      </c>
+      <c r="J40" s="12" t="n">
+        <v>2020</v>
+      </c>
+      <c r="K40" s="12" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="41" ht="38" customHeight="1">
       <c r="A41" s="12" t="inlineStr">
         <is>
           <t>BSD-01+BSD-MB-06-V7</t>
@@ -1906,7 +2353,7 @@
       </c>
       <c r="B41" s="13" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes CLE W236 2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Unghi mort Mercedes CLE W236 2024 - Sistem BSD cu oglinzi dedicate</t>
         </is>
       </c>
       <c r="C41" s="12" t="inlineStr"/>
@@ -1926,13 +2373,24 @@
           <t>Mercedes-Benz</t>
         </is>
       </c>
-      <c r="H41" s="13" t="inlineStr">
-        <is>
-          <t>CLE (W236) 2024</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="40" customHeight="1">
+      <c r="H41" s="12" t="inlineStr">
+        <is>
+          <t>CLE</t>
+        </is>
+      </c>
+      <c r="I41" s="12" t="inlineStr">
+        <is>
+          <t>W236</t>
+        </is>
+      </c>
+      <c r="J41" s="12" t="n">
+        <v>2023</v>
+      </c>
+      <c r="K41" s="12" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="42" ht="38" customHeight="1">
       <c r="A42" s="14" t="inlineStr">
         <is>
           <t>BSD-01+BSD-MB-07-V1</t>
@@ -1940,7 +2398,7 @@
       </c>
       <c r="B42" s="15" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes GLE W167 2020-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Unghi mort Mercedes GLE W167 2020-2024 - Sistem BSD cu oglinzi dedicate</t>
         </is>
       </c>
       <c r="C42" s="14" t="inlineStr"/>
@@ -1960,13 +2418,24 @@
           <t>Mercedes-Benz</t>
         </is>
       </c>
-      <c r="H42" s="15" t="inlineStr">
-        <is>
-          <t>GLE (W167) 2020-2024</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="40" customHeight="1">
+      <c r="H42" s="14" t="inlineStr">
+        <is>
+          <t>GLE</t>
+        </is>
+      </c>
+      <c r="I42" s="14" t="inlineStr">
+        <is>
+          <t>V167</t>
+        </is>
+      </c>
+      <c r="J42" s="14" t="n">
+        <v>2018</v>
+      </c>
+      <c r="K42" s="14" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="43" ht="38" customHeight="1">
       <c r="A43" s="14" t="inlineStr">
         <is>
           <t>BSD-01+BSD-MB-07-V2</t>
@@ -1974,7 +2443,7 @@
       </c>
       <c r="B43" s="15" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes GLS X167 2020-2024 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Unghi mort Mercedes GLS X167 2020-2024 - Sistem BSD cu oglinzi dedicate</t>
         </is>
       </c>
       <c r="C43" s="14" t="inlineStr"/>
@@ -1994,13 +2463,24 @@
           <t>Mercedes-Benz</t>
         </is>
       </c>
-      <c r="H43" s="15" t="inlineStr">
-        <is>
-          <t>GLS (X167) 2020-2024</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="40" customHeight="1">
+      <c r="H43" s="14" t="inlineStr">
+        <is>
+          <t>GLS</t>
+        </is>
+      </c>
+      <c r="I43" s="14" t="inlineStr">
+        <is>
+          <t>X167</t>
+        </is>
+      </c>
+      <c r="J43" s="14" t="n">
+        <v>2019</v>
+      </c>
+      <c r="K43" s="14" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="44" ht="38" customHeight="1">
       <c r="A44" s="14" t="inlineStr">
         <is>
           <t>BSD-01+BSD-MB-07-V3</t>
@@ -2008,7 +2488,7 @@
       </c>
       <c r="B44" s="15" t="inlineStr">
         <is>
-          <t>Unghi mort Mercedes G-Class W463 2019-2022 - Sistem BSD dedicat cu oglinzi</t>
+          <t>Unghi mort Mercedes G-Class W463 2019-2022 - Sistem BSD cu oglinzi dedicate</t>
         </is>
       </c>
       <c r="C44" s="14" t="inlineStr"/>
@@ -2028,10 +2508,21 @@
           <t>Mercedes-Benz</t>
         </is>
       </c>
-      <c r="H44" s="15" t="inlineStr">
-        <is>
-          <t>G-Class (W463) 2019-2022</t>
-        </is>
+      <c r="H44" s="14" t="inlineStr">
+        <is>
+          <t>G-Class</t>
+        </is>
+      </c>
+      <c r="I44" s="14" t="inlineStr">
+        <is>
+          <t>W463</t>
+        </is>
+      </c>
+      <c r="J44" s="14" t="n">
+        <v>2018</v>
+      </c>
+      <c r="K44" s="14" t="n">
+        <v>2026</v>
       </c>
     </row>
   </sheetData>

</xml_diff>